<commit_message>
fix: add Tester column to test cases; add migration 029 for invite token constraint
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases/Zawaaj_Test_Cases.xlsx
+++ b/test-cases/Zawaaj_Test_Cases.xlsx
@@ -402,17 +402,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:J30"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="38.83203125" customWidth="1"/>
-    <col min="4" max="4" width="32.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
     <col min="6" max="6" width="48.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="48.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -420,27 +421,30 @@
         <v>Test ID</v>
       </c>
       <c r="B1" t="str">
+        <v>Tester</v>
+      </c>
+      <c r="C1" t="str">
         <v>Category</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Test Case</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Pre-conditions</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Steps</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Expected Behaviour</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Actual Behaviour</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Pass / Fail</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -449,29 +453,32 @@
         <v>MEM-001</v>
       </c>
       <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
         <v>Login</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Sign in with valid credentials</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Approved member account exists</v>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
+      <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Go to zawaaj.uk/login
 2. Enter email and password
 3. Click Sign in</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Redirect to /browse; sidebar shows member name and avatar</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v/>
       </c>
     </row>
@@ -480,29 +487,32 @@
         <v>MEM-002</v>
       </c>
       <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
         <v>Login</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Sign in with wrong password</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Account exists</v>
       </c>
-      <c r="E3" t="str" xml:space="preserve">
+      <c r="F3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Go to /login
 2. Enter correct email, wrong password
 3. Click Sign in</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>Error message displayed; user remains on login page</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
       <c r="H3" t="str">
         <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v/>
       </c>
     </row>
@@ -511,31 +521,34 @@
         <v>MEM-003</v>
       </c>
       <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
         <v>Login</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Forgot password — reset email flow</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Account exists</v>
       </c>
-      <c r="E4" t="str" xml:space="preserve">
+      <c r="F4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click "Forgot password"
 2. Enter email
 3. Click send
 4. Open email, click link
 5. Enter new password</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Password updated; redirected to /browse</v>
       </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
         <v/>
       </c>
     </row>
@@ -544,27 +557,30 @@
         <v>MEM-004</v>
       </c>
       <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
         <v>Browse</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>View browse page — approved profiles only</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>Signed in as approved member</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>1. Navigate to /browse</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>Grid of opposite-gender approved profiles shown; own profile not visible</v>
       </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
       <c r="H5" t="str">
         <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v/>
       </c>
     </row>
@@ -573,29 +589,32 @@
         <v>MEM-005</v>
       </c>
       <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
         <v>Browse</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>Apply school of thought filter</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>On /browse</v>
       </c>
-      <c r="E6" t="str" xml:space="preserve">
+      <c r="F6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open filter panel
 2. Select a school of thought
 3. Apply</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>Grid refreshes; only profiles matching selection shown</v>
       </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
         <v/>
       </c>
     </row>
@@ -604,29 +623,32 @@
         <v>MEM-006</v>
       </c>
       <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
         <v>Browse</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>Apply location filter</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>On /browse</v>
       </c>
-      <c r="E7" t="str" xml:space="preserve">
+      <c r="F7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open filter panel
 2. Type/select a location
 3. Apply</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>Grid refreshes showing only matching locations</v>
       </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
       <c r="H7" t="str">
         <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
         <v/>
       </c>
     </row>
@@ -635,27 +657,30 @@
         <v>MEM-007</v>
       </c>
       <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
         <v>Browse</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>New profile badge</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>On /browse; a profile was approved recently</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>1. Browse grid</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>"New" gold badge visible on profiles listed within the last 7 days</v>
       </c>
-      <c r="G8" t="str">
-        <v/>
-      </c>
       <c r="H8" t="str">
         <v/>
       </c>
       <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
         <v/>
       </c>
     </row>
@@ -664,27 +689,30 @@
         <v>MEM-008</v>
       </c>
       <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
         <v>Browse</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>Search by initials / name</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>On /browse</v>
       </c>
-      <c r="E9" t="str">
+      <c r="F9" t="str">
         <v>1. Type initials into search box</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>Grid filters in real-time to matching profiles</v>
       </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
       <c r="H9" t="str">
         <v/>
       </c>
       <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
         <v/>
       </c>
     </row>
@@ -693,27 +721,30 @@
         <v>MEM-009</v>
       </c>
       <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
         <v>Profile view</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>Open profile modal from browse card</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>On /browse</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>1. Click a profile card</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>Slide panel opens with full profile details; compatibility bar visible</v>
       </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
       <c r="H10" t="str">
         <v/>
       </c>
       <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
         <v/>
       </c>
     </row>
@@ -722,27 +753,30 @@
         <v>MEM-010</v>
       </c>
       <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
         <v>Profile view</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>Full profile details locked for free tier</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>Free plan account; viewing another profile</v>
       </c>
-      <c r="E11" t="str">
+      <c r="F11" t="str">
         <v>1. Open profile modal</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>Faith &amp; values section blurred with "Upgrade to Premium" overlay</v>
       </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
       <c r="H11" t="str">
         <v/>
       </c>
       <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
         <v/>
       </c>
     </row>
@@ -751,27 +785,30 @@
         <v>MEM-011</v>
       </c>
       <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
         <v>Profile view</v>
       </c>
-      <c r="C12" t="str">
+      <c r="D12" t="str">
         <v>Full profile visible for Premium</v>
       </c>
-      <c r="D12" t="str">
+      <c r="E12" t="str">
         <v>Premium plan account</v>
       </c>
-      <c r="E12" t="str">
+      <c r="F12" t="str">
         <v>1. Open profile modal</v>
       </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
         <v>Full faith details, bio, preferences all visible</v>
       </c>
-      <c r="G12" t="str">
-        <v/>
-      </c>
       <c r="H12" t="str">
         <v/>
       </c>
       <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
         <v/>
       </c>
     </row>
@@ -780,29 +817,32 @@
         <v>MEM-012</v>
       </c>
       <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C13" t="str">
+      <c r="D13" t="str">
         <v>Express interest in a profile</v>
       </c>
-      <c r="D13" t="str">
+      <c r="E13" t="str">
         <v>Approved member; monthly limit not reached; no existing request</v>
       </c>
-      <c r="E13" t="str" xml:space="preserve">
+      <c r="F13" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open a profile modal
 2. Click "Express interest"
 3. Click Confirm</v>
       </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
         <v>Toast/confirmation shown; button changes to "Interest sent ✓"; count incremented</v>
       </c>
-      <c r="G13" t="str">
-        <v/>
-      </c>
       <c r="H13" t="str">
         <v/>
       </c>
       <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
         <v/>
       </c>
     </row>
@@ -811,28 +851,31 @@
         <v>MEM-013</v>
       </c>
       <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C14" t="str">
+      <c r="D14" t="str">
         <v>Monthly limit enforced</v>
       </c>
-      <c r="D14" t="str">
+      <c r="E14" t="str">
         <v>Member has used all monthly interest expressions</v>
       </c>
-      <c r="E14" t="str" xml:space="preserve">
+      <c r="F14" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open a profile modal
 2. Attempt to express interest</v>
       </c>
-      <c r="F14" t="str">
+      <c r="G14" t="str">
         <v>Button shows "Monthly limit reached"; cannot proceed; upgrade prompt shown for free users</v>
       </c>
-      <c r="G14" t="str">
-        <v/>
-      </c>
       <c r="H14" t="str">
         <v/>
       </c>
       <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
         <v/>
       </c>
     </row>
@@ -841,27 +884,30 @@
         <v>MEM-014</v>
       </c>
       <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C15" t="str">
+      <c r="D15" t="str">
         <v>View sent introductions</v>
       </c>
-      <c r="D15" t="str">
+      <c r="E15" t="str">
         <v>At least one request sent</v>
       </c>
-      <c r="E15" t="str">
+      <c r="F15" t="str">
         <v>1. Navigate to /introductions</v>
       </c>
-      <c r="F15" t="str">
+      <c r="G15" t="str">
         <v>List of sent requests with status badges (Pending / Accepted / Declined / Expired)</v>
       </c>
-      <c r="G15" t="str">
-        <v/>
-      </c>
       <c r="H15" t="str">
         <v/>
       </c>
       <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
         <v/>
       </c>
     </row>
@@ -870,28 +916,31 @@
         <v>MEM-015</v>
       </c>
       <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C16" t="str">
+      <c r="D16" t="str">
         <v>View received introduction requests</v>
       </c>
-      <c r="D16" t="str">
+      <c r="E16" t="str">
         <v>Member has received a pending request</v>
       </c>
-      <c r="E16" t="str" xml:space="preserve">
+      <c r="F16" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to /introductions
 2. Check "Received" tab</v>
       </c>
-      <c r="F16" t="str">
+      <c r="G16" t="str">
         <v>Pending request card visible with Accept / Decline option (free) or template selection (Premium)</v>
       </c>
-      <c r="G16" t="str">
-        <v/>
-      </c>
       <c r="H16" t="str">
         <v/>
       </c>
       <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
         <v/>
       </c>
     </row>
@@ -900,28 +949,31 @@
         <v>MEM-016</v>
       </c>
       <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C17" t="str">
+      <c r="D17" t="str">
         <v>Accept a received request</v>
       </c>
-      <c r="D17" t="str">
+      <c r="E17" t="str">
         <v>Pending request in received tab</v>
       </c>
-      <c r="E17" t="str" xml:space="preserve">
+      <c r="F17" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click Accept on a received request
 2. Confirm</v>
       </c>
-      <c r="F17" t="str">
+      <c r="G17" t="str">
         <v>Status changes to Accepted; match created; in-app notification shown; both families receive email</v>
       </c>
-      <c r="G17" t="str">
-        <v/>
-      </c>
       <c r="H17" t="str">
         <v/>
       </c>
       <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
         <v/>
       </c>
     </row>
@@ -930,28 +982,31 @@
         <v>MEM-017</v>
       </c>
       <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C18" t="str">
+      <c r="D18" t="str">
         <v>Decline a received request</v>
       </c>
-      <c r="D18" t="str">
+      <c r="E18" t="str">
         <v>Pending request in received tab</v>
       </c>
-      <c r="E18" t="str" xml:space="preserve">
+      <c r="F18" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click Decline
 2. Confirm</v>
       </c>
-      <c r="F18" t="str">
+      <c r="G18" t="str">
         <v>Status changes to Declined; sensitive decline notification sent to sender; no email</v>
       </c>
-      <c r="G18" t="str">
-        <v/>
-      </c>
       <c r="H18" t="str">
         <v/>
       </c>
       <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
         <v/>
       </c>
     </row>
@@ -960,27 +1015,30 @@
         <v>MEM-018</v>
       </c>
       <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
         <v>Shortlist</v>
       </c>
-      <c r="C19" t="str">
+      <c r="D19" t="str">
         <v>Save a profile to shortlist</v>
       </c>
-      <c r="D19" t="str">
+      <c r="E19" t="str">
         <v>Viewing a profile modal</v>
       </c>
-      <c r="E19" t="str">
+      <c r="F19" t="str">
         <v>1. Click the heart icon on a profile</v>
       </c>
-      <c r="F19" t="str">
+      <c r="G19" t="str">
         <v>Heart filled; profile appears in shortlist tab; count updated in sidebar</v>
       </c>
-      <c r="G19" t="str">
-        <v/>
-      </c>
       <c r="H19" t="str">
         <v/>
       </c>
       <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
         <v/>
       </c>
     </row>
@@ -989,27 +1047,30 @@
         <v>MEM-019</v>
       </c>
       <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
         <v>Shortlist</v>
       </c>
-      <c r="C20" t="str">
+      <c r="D20" t="str">
         <v>Remove from shortlist</v>
       </c>
-      <c r="D20" t="str">
+      <c r="E20" t="str">
         <v>Profile is saved</v>
       </c>
-      <c r="E20" t="str">
+      <c r="F20" t="str">
         <v>1. Click filled heart icon again</v>
       </c>
-      <c r="F20" t="str">
+      <c r="G20" t="str">
         <v>Profile removed from shortlist; count decremented</v>
       </c>
-      <c r="G20" t="str">
-        <v/>
-      </c>
       <c r="H20" t="str">
         <v/>
       </c>
       <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
         <v/>
       </c>
     </row>
@@ -1018,27 +1079,30 @@
         <v>MEM-020</v>
       </c>
       <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
         <v>My Profile</v>
       </c>
-      <c r="C21" t="str">
+      <c r="D21" t="str">
         <v>View own profile</v>
       </c>
-      <c r="D21" t="str">
+      <c r="E21" t="str">
         <v>Signed in as approved member</v>
       </c>
-      <c r="E21" t="str">
+      <c r="F21" t="str">
         <v>1. Navigate to /my-profile</v>
       </c>
-      <c r="F21" t="str">
+      <c r="G21" t="str">
         <v>Own profile details displayed in read-only view</v>
       </c>
-      <c r="G21" t="str">
-        <v/>
-      </c>
       <c r="H21" t="str">
         <v/>
       </c>
       <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
         <v/>
       </c>
     </row>
@@ -1047,29 +1111,32 @@
         <v>MEM-021</v>
       </c>
       <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22" t="str">
         <v>My Profile</v>
       </c>
-      <c r="C22" t="str">
+      <c r="D22" t="str">
         <v>Edit basic info</v>
       </c>
-      <c r="D22" t="str">
+      <c r="E22" t="str">
         <v>On /my-profile</v>
       </c>
-      <c r="E22" t="str" xml:space="preserve">
+      <c r="F22" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click Edit
 2. Update location or profession
 3. Save</v>
       </c>
-      <c r="F22" t="str">
+      <c r="G22" t="str">
         <v>Changes saved; profile updated immediately</v>
       </c>
-      <c r="G22" t="str">
-        <v/>
-      </c>
       <c r="H22" t="str">
         <v/>
       </c>
       <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
         <v/>
       </c>
     </row>
@@ -1078,29 +1145,32 @@
         <v>MEM-022</v>
       </c>
       <c r="B23" t="str">
+        <v/>
+      </c>
+      <c r="C23" t="str">
         <v>My Profile</v>
       </c>
-      <c r="C23" t="str">
+      <c r="D23" t="str">
         <v>Edit faith fields (female — niqab, abaya)</v>
       </c>
-      <c r="D23" t="str">
+      <c r="E23" t="str">
         <v>Signed in as female member; on /my-profile</v>
       </c>
-      <c r="E23" t="str" xml:space="preserve">
+      <c r="F23" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click Edit
 2. Select niqab and abaya options
 3. Save</v>
       </c>
-      <c r="F23" t="str">
+      <c r="G23" t="str">
         <v>Values saved; displayed in faith section on own profile and profile view for Premium viewers</v>
       </c>
-      <c r="G23" t="str">
-        <v/>
-      </c>
       <c r="H23" t="str">
         <v/>
       </c>
       <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
         <v/>
       </c>
     </row>
@@ -1109,29 +1179,32 @@
         <v>MEM-023</v>
       </c>
       <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
         <v>My Profile</v>
       </c>
-      <c r="C24" t="str">
+      <c r="D24" t="str">
         <v>Edit Quran engagement (all genders)</v>
       </c>
-      <c r="D24" t="str">
+      <c r="E24" t="str">
         <v>On /my-profile</v>
       </c>
-      <c r="E24" t="str" xml:space="preserve">
+      <c r="F24" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click Edit
 2. Select Quran engagement level
 3. Save</v>
       </c>
-      <c r="F24" t="str">
+      <c r="G24" t="str">
         <v>Value saved and displayed in faith section</v>
       </c>
-      <c r="G24" t="str">
-        <v/>
-      </c>
       <c r="H24" t="str">
         <v/>
       </c>
       <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
         <v/>
       </c>
     </row>
@@ -1140,27 +1213,30 @@
         <v>MEM-024</v>
       </c>
       <c r="B25" t="str">
+        <v/>
+      </c>
+      <c r="C25" t="str">
         <v>My Profile</v>
       </c>
-      <c r="C25" t="str">
+      <c r="D25" t="str">
         <v>Pause profile</v>
       </c>
-      <c r="D25" t="str">
+      <c r="E25" t="str">
         <v>Approved member on /my-profile</v>
       </c>
-      <c r="E25" t="str">
+      <c r="F25" t="str">
         <v>1. Click "Pause my profile"</v>
       </c>
-      <c r="F25" t="str">
+      <c r="G25" t="str">
         <v>Confirmation prompt shown; on confirm: profile status → paused; no longer visible in browse</v>
       </c>
-      <c r="G25" t="str">
-        <v/>
-      </c>
       <c r="H25" t="str">
         <v/>
       </c>
       <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
         <v/>
       </c>
     </row>
@@ -1169,29 +1245,32 @@
         <v>MEM-025</v>
       </c>
       <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
         <v>My Profile</v>
       </c>
-      <c r="C26" t="str">
+      <c r="D26" t="str">
         <v>Withdraw profile</v>
       </c>
-      <c r="D26" t="str">
+      <c r="E26" t="str">
         <v>Approved member on /my-profile</v>
       </c>
-      <c r="E26" t="str" xml:space="preserve">
+      <c r="F26" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click "Withdraw my profile"
 2. Select reason
 3. Confirm</v>
       </c>
-      <c r="F26" t="str">
+      <c r="G26" t="str">
         <v>Profile withdrawn; member logged out or redirected to pending page</v>
       </c>
-      <c r="G26" t="str">
-        <v/>
-      </c>
       <c r="H26" t="str">
         <v/>
       </c>
       <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
         <v/>
       </c>
     </row>
@@ -1200,27 +1279,30 @@
         <v>MEM-026</v>
       </c>
       <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
         <v>Events</v>
       </c>
-      <c r="C27" t="str">
+      <c r="D27" t="str">
         <v>View upcoming events</v>
       </c>
-      <c r="D27" t="str">
+      <c r="E27" t="str">
         <v>Approved member</v>
       </c>
-      <c r="E27" t="str">
+      <c r="F27" t="str">
         <v>1. Navigate to /events</v>
       </c>
-      <c r="F27" t="str">
+      <c r="G27" t="str">
         <v>Upcoming events listed with date, location, registration link</v>
       </c>
-      <c r="G27" t="str">
-        <v/>
-      </c>
       <c r="H27" t="str">
         <v/>
       </c>
       <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
         <v/>
       </c>
     </row>
@@ -1229,27 +1311,30 @@
         <v>MEM-027</v>
       </c>
       <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
         <v>Events</v>
       </c>
-      <c r="C28" t="str">
+      <c r="D28" t="str">
         <v>Register for event via external link</v>
       </c>
-      <c r="D28" t="str">
+      <c r="E28" t="str">
         <v>Upcoming event with registration URL</v>
       </c>
-      <c r="E28" t="str">
+      <c r="F28" t="str">
         <v>1. Click "Register →" on event card</v>
       </c>
-      <c r="F28" t="str">
+      <c r="G28" t="str">
         <v>External registration page opens in new tab</v>
       </c>
-      <c r="G28" t="str">
-        <v/>
-      </c>
       <c r="H28" t="str">
         <v/>
       </c>
       <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
         <v/>
       </c>
     </row>
@@ -1258,28 +1343,31 @@
         <v>MEM-028</v>
       </c>
       <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
         <v>Pending state</v>
       </c>
-      <c r="C29" t="str">
+      <c r="D29" t="str">
         <v>New signup — pending approval view</v>
       </c>
-      <c r="D29" t="str">
+      <c r="E29" t="str">
         <v>Registered but admin has not approved yet</v>
       </c>
-      <c r="E29" t="str" xml:space="preserve">
+      <c r="F29" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Complete signup
 2. Check /pending page</v>
       </c>
-      <c r="F29" t="str">
+      <c r="G29" t="str">
         <v>Clock icon shown with "Application submitted" message and sign-out link</v>
       </c>
-      <c r="G29" t="str">
-        <v/>
-      </c>
       <c r="H29" t="str">
         <v/>
       </c>
       <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
         <v/>
       </c>
     </row>
@@ -1288,50 +1376,54 @@
         <v>MEM-029</v>
       </c>
       <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
         <v>Pending state</v>
       </c>
-      <c r="C30" t="str">
+      <c r="D30" t="str">
         <v>Email verification pending state</v>
       </c>
-      <c r="D30" t="str">
+      <c r="E30" t="str">
         <v>Account created but email not verified</v>
       </c>
-      <c r="E30" t="str">
+      <c r="F30" t="str">
         <v>1. Check /pending page</v>
       </c>
-      <c r="F30" t="str">
+      <c r="G30" t="str">
         <v>Envelope icon shown; contact email displayed; "Resend verification" button available</v>
       </c>
-      <c r="G30" t="str">
-        <v/>
-      </c>
       <c r="H30" t="str">
         <v/>
       </c>
       <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J30"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:J14"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="38.83203125" customWidth="1"/>
-    <col min="4" max="4" width="32.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
     <col min="6" max="6" width="48.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="48.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1339,27 +1431,30 @@
         <v>Test ID</v>
       </c>
       <c r="B1" t="str">
+        <v>Tester</v>
+      </c>
+      <c r="C1" t="str">
         <v>Category</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Test Case</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Pre-conditions</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Steps</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Expected Behaviour</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Actual Behaviour</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Pass / Fail</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -1368,28 +1463,31 @@
         <v>MGR-001</v>
       </c>
       <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
         <v>Login</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Manager sign in</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Manager account exists with role = manager</v>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
+      <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Go to /login
 2. Sign in with manager credentials</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Redirect to /admin/introductions (not full dashboard)</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v/>
       </c>
     </row>
@@ -1398,27 +1496,30 @@
         <v>MGR-002</v>
       </c>
       <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>View introduction requests list</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Signed in as manager</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>1. Navigate to /admin/introductions</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>All introduction requests visible with filters for status</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
       <c r="H3" t="str">
         <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v/>
       </c>
     </row>
@@ -1427,28 +1528,31 @@
         <v>MGR-003</v>
       </c>
       <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Filter introductions by status</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>On admin introductions page</v>
       </c>
-      <c r="E4" t="str" xml:space="preserve">
+      <c r="F4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Select "Pending" filter
 2. Then try "Accepted"</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Table updates to show only requests matching selected status</v>
       </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
         <v/>
       </c>
     </row>
@@ -1457,27 +1561,30 @@
         <v>MGR-004</v>
       </c>
       <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>Search introduction requests</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>On admin introductions page</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>1. Type member name or initials in search</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>Results filter in real-time</v>
       </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
       <c r="H5" t="str">
         <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v/>
       </c>
     </row>
@@ -1486,27 +1593,30 @@
         <v>MGR-005</v>
       </c>
       <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>View introduction request detail</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>On admin introductions page</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>1. Click a request row</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>Side panel opens with profile A and profile B details, request status, timestamps</v>
       </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
         <v/>
       </c>
     </row>
@@ -1515,29 +1625,32 @@
         <v>MGR-006</v>
       </c>
       <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>Update introduction request status</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>Accepted mutual request visible</v>
       </c>
-      <c r="E7" t="str" xml:space="preserve">
+      <c r="F7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open request detail
 2. Change status to "Facilitated"
 3. Save</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>Status updated; both member profiles show "Contacts shared" badge</v>
       </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
       <c r="H7" t="str">
         <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
         <v/>
       </c>
     </row>
@@ -1546,29 +1659,32 @@
         <v>MGR-007</v>
       </c>
       <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
         <v>Introductions</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>Record outcome on an introduction</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>Facilitated request</v>
       </c>
-      <c r="E8" t="str" xml:space="preserve">
+      <c r="F8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open request detail
 2. Set outcome (e.g. "In conversation")
 3. Save</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>Outcome recorded with timestamp; visible in admin view</v>
       </c>
-      <c r="G8" t="str">
-        <v/>
-      </c>
       <c r="H8" t="str">
         <v/>
       </c>
       <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
         <v/>
       </c>
     </row>
@@ -1577,27 +1693,30 @@
         <v>MGR-008</v>
       </c>
       <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
         <v>Profile</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>View any member profile (admin view)</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>Signed in as manager</v>
       </c>
-      <c r="E9" t="str">
+      <c r="F9" t="str">
         <v>1. Navigate to /admin/profile/[id]</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>Full profile including sensitive fields (contact number, date of birth, admin notes)</v>
       </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
       <c r="H9" t="str">
         <v/>
       </c>
       <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
         <v/>
       </c>
     </row>
@@ -1606,28 +1725,31 @@
         <v>MGR-009</v>
       </c>
       <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
         <v>Profile</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>Approve a pending profile</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>Profile with status = pending</v>
       </c>
-      <c r="E10" t="str" xml:space="preserve">
+      <c r="F10" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open admin profile view
 2. Click Approve</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>Profile status → approved; listed_at set; member appears in browse</v>
       </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
       <c r="H10" t="str">
         <v/>
       </c>
       <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
         <v/>
       </c>
     </row>
@@ -1636,28 +1758,31 @@
         <v>MGR-010</v>
       </c>
       <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
         <v>Profile</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>Reject a pending profile</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>Profile with status = pending</v>
       </c>
-      <c r="E11" t="str" xml:space="preserve">
+      <c r="F11" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open admin profile view
 2. Click Reject</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>Profile status → rejected; member sees rejection on /pending</v>
       </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
       <c r="H11" t="str">
         <v/>
       </c>
       <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
         <v/>
       </c>
     </row>
@@ -1666,28 +1791,31 @@
         <v>MGR-011</v>
       </c>
       <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
         <v>Profile</v>
       </c>
-      <c r="C12" t="str">
+      <c r="D12" t="str">
         <v>Suspend an active profile</v>
       </c>
-      <c r="D12" t="str">
+      <c r="E12" t="str">
         <v>Approved profile</v>
       </c>
-      <c r="E12" t="str" xml:space="preserve">
+      <c r="F12" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Open admin profile view
 2. Click Suspend</v>
       </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
         <v>Profile status → suspended; disappears from browse; member cannot access member pages</v>
       </c>
-      <c r="G12" t="str">
-        <v/>
-      </c>
       <c r="H12" t="str">
         <v/>
       </c>
       <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
         <v/>
       </c>
     </row>
@@ -1696,29 +1824,32 @@
         <v>MGR-012</v>
       </c>
       <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
         <v>Profile</v>
       </c>
-      <c r="C13" t="str">
+      <c r="D13" t="str">
         <v>Add admin notes to a profile</v>
       </c>
-      <c r="D13" t="str">
+      <c r="E13" t="str">
         <v>On any admin profile view</v>
       </c>
-      <c r="E13" t="str" xml:space="preserve">
+      <c r="F13" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click "Edit admin notes"
 2. Type notes
 3. Save</v>
       </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
         <v>Notes saved and visible only to admin/managers; not visible to member</v>
       </c>
-      <c r="G13" t="str">
-        <v/>
-      </c>
       <c r="H13" t="str">
         <v/>
       </c>
       <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
         <v/>
       </c>
     </row>
@@ -1727,52 +1858,56 @@
         <v>MGR-013</v>
       </c>
       <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
         <v>Email</v>
       </c>
-      <c r="C14" t="str">
+      <c r="D14" t="str">
         <v>Send admin message email to a family</v>
       </c>
-      <c r="D14" t="str">
+      <c r="E14" t="str">
         <v>On admin families page</v>
       </c>
-      <c r="E14" t="str" xml:space="preserve">
+      <c r="F14" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click "✉ Email family" next to a family
 2. Enter subject and message
 3. Send</v>
       </c>
-      <c r="F14" t="str">
+      <c r="G14" t="str">
         <v>Email sent via Resend to family contact email; success confirmation shown</v>
       </c>
-      <c r="G14" t="str">
-        <v/>
-      </c>
       <c r="H14" t="str">
         <v/>
       </c>
       <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J14"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:J12"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="38.83203125" customWidth="1"/>
-    <col min="4" max="4" width="32.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
     <col min="6" max="6" width="48.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="48.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1780,27 +1915,30 @@
         <v>Test ID</v>
       </c>
       <c r="B1" t="str">
+        <v>Tester</v>
+      </c>
+      <c r="C1" t="str">
         <v>Category</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Test Case</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Pre-conditions</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Steps</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Expected Behaviour</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Actual Behaviour</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Pass / Fail</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -1809,29 +1947,32 @@
         <v>PAR-A-001</v>
       </c>
       <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
         <v>Registration</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Check email uniqueness at step 0</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>No existing account with email</v>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
+      <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Go to /register
 2. Enter email
 3. Click Next</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Proceeds to step 1; no error</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v/>
       </c>
     </row>
@@ -1840,29 +1981,32 @@
         <v>PAR-A-002</v>
       </c>
       <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
         <v>Registration</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Email already taken at step 0</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Email exists in auth.users</v>
       </c>
-      <c r="E3" t="str" xml:space="preserve">
+      <c r="F3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Go to /register
 2. Enter existing email
 3. Click Next</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>Error: "An account with this email already exists." — cannot proceed</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
       <c r="H3" t="str">
         <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v/>
       </c>
     </row>
@@ -1871,27 +2015,30 @@
         <v>PAR-A-003</v>
       </c>
       <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
         <v>Registration</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Complete 8-step registration wizard — candidate details</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Valid email; no existing account</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>1. Complete steps 1-3: candidate personal info (name, DOB, location, profession, education, faith, bio)</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Form validates each step before allowing Next</v>
       </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
         <v/>
       </c>
     </row>
@@ -1900,27 +2047,30 @@
         <v>PAR-A-004</v>
       </c>
       <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
         <v>Registration</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>Guardian / contact details step (step 4)</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>No invite token; continuing registration</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>1. Complete step 4: guardian name, contact number, relationship</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>Guardian fields required; cannot skip</v>
       </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
       <c r="H5" t="str">
         <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v/>
       </c>
     </row>
@@ -1929,27 +2079,30 @@
         <v>PAR-A-005</v>
       </c>
       <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
         <v>Registration</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>Preferences step</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>On step 5</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>1. Complete partner preferences (age range, location, school of thought, ethnicity)</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>All fields optional; can proceed without selecting</v>
       </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
         <v/>
       </c>
     </row>
@@ -1958,28 +2111,31 @@
         <v>PAR-A-006</v>
       </c>
       <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
         <v>Registration</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>Terms &amp; consent step</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>On step 7</v>
       </c>
-      <c r="E7" t="str" xml:space="preserve">
+      <c r="F7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Check consent and terms boxes
 2. Click Submit</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>Cannot submit without both boxes checked</v>
       </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
       <c r="H7" t="str">
         <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
         <v/>
       </c>
     </row>
@@ -1988,27 +2144,30 @@
         <v>PAR-A-007</v>
       </c>
       <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
         <v>Registration</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>Successful registration</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>All steps complete; valid data</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>1. Click Submit on final step</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>Account created; family account created; profile created with status=pending; redirect to /pending</v>
       </c>
-      <c r="G8" t="str">
-        <v/>
-      </c>
       <c r="H8" t="str">
         <v/>
       </c>
       <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
         <v/>
       </c>
     </row>
@@ -2017,27 +2176,30 @@
         <v>PAR-A-008</v>
       </c>
       <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
         <v>Post-registration</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>Pending page after registration</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>Just completed registration</v>
       </c>
-      <c r="E9" t="str">
+      <c r="F9" t="str">
         <v>1. After redirect to /pending</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>Clock icon shown; "Application submitted — JazakAllahu Khayran" message; sign-out link</v>
       </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
       <c r="H9" t="str">
         <v/>
       </c>
       <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
         <v/>
       </c>
     </row>
@@ -2046,28 +2208,31 @@
         <v>PAR-A-009</v>
       </c>
       <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
         <v>Post-registration</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>Profile not visible in browse before approval</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>Profile status = pending</v>
       </c>
-      <c r="E10" t="str" xml:space="preserve">
+      <c r="F10" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in as another member
 2. Browse member directory</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>Newly registered profile not visible</v>
       </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
       <c r="H10" t="str">
         <v/>
       </c>
       <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
         <v/>
       </c>
     </row>
@@ -2076,27 +2241,30 @@
         <v>PAR-A-010</v>
       </c>
       <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
         <v>Family account</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>Family account created on registration</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>Completed Path A registration</v>
       </c>
-      <c r="E11" t="str">
+      <c r="F11" t="str">
         <v>1. In Supabase / admin families view, search by contact email</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>Family account row exists with contact_full_name, contact_email, registration_path = direct</v>
       </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
       <c r="H11" t="str">
         <v/>
       </c>
       <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
         <v/>
       </c>
     </row>
@@ -2105,51 +2273,55 @@
         <v>PAR-A-011</v>
       </c>
       <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
         <v>Family account</v>
       </c>
-      <c r="C12" t="str">
+      <c r="D12" t="str">
         <v>Admin can view family details after Path A</v>
       </c>
-      <c r="D12" t="str">
+      <c r="E12" t="str">
         <v>As admin; on /admin/families</v>
       </c>
-      <c r="E12" t="str" xml:space="preserve">
+      <c r="F12" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Search for family
 2. Open family row</v>
       </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
         <v>Contact details, family members, invite tokens all visible</v>
       </c>
-      <c r="G12" t="str">
-        <v/>
-      </c>
       <c r="H12" t="str">
         <v/>
       </c>
       <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:J7"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="38.83203125" customWidth="1"/>
-    <col min="4" max="4" width="32.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
     <col min="6" max="6" width="48.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="48.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2157,27 +2329,30 @@
         <v>Test ID</v>
       </c>
       <c r="B1" t="str">
+        <v>Tester</v>
+      </c>
+      <c r="C1" t="str">
         <v>Category</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Test Case</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Pre-conditions</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Steps</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Expected Behaviour</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Actual Behaviour</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Pass / Fail</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -2186,27 +2361,30 @@
         <v>CHD-B-001</v>
       </c>
       <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
         <v>Registration</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Child navigates to /register/child</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>No invite token; child wants to register independently</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>1. Go to /register/child</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Multi-step form loads; no token banner; all steps including guardian step present</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v/>
       </c>
     </row>
@@ -2215,27 +2393,30 @@
         <v>CHD-B-002</v>
       </c>
       <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
         <v>Registration</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>All steps present without invite token</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>On /register/child with no ?token= param</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>1. Step through form</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>8 steps shown including Guardian contact details step (step 4)</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
       <c r="H3" t="str">
         <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v/>
       </c>
     </row>
@@ -2244,28 +2425,31 @@
         <v>CHD-B-003</v>
       </c>
       <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
         <v>Registration</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Guardian/contact details required (Path B direct)</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>On step 4 of child registration</v>
       </c>
-      <c r="E4" t="str" xml:space="preserve">
+      <c r="F4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Leave guardian fields blank
 2. Try to proceed</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Validation error; cannot proceed without guardian contact info</v>
       </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
         <v/>
       </c>
     </row>
@@ -2274,28 +2458,31 @@
         <v>CHD-B-004</v>
       </c>
       <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
         <v>Registration</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>Complete child registration — independent</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>Valid email; no existing account</v>
       </c>
-      <c r="E5" t="str" xml:space="preserve">
+      <c r="F5" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Complete all 8 steps with guardian details
 2. Submit</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>Auth user created; new family account created; profile created; redirect to /pending</v>
       </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
       <c r="H5" t="str">
         <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v/>
       </c>
     </row>
@@ -2304,27 +2491,30 @@
         <v>CHD-B-005</v>
       </c>
       <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
         <v>Post-registration</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>Pending state after child direct registration</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>Just completed child Path B registration</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>1. Check /pending</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>"Application submitted" message with clock icon; no email verification pending state</v>
       </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
         <v/>
       </c>
     </row>
@@ -2333,50 +2523,54 @@
         <v>CHD-B-006</v>
       </c>
       <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
         <v>Family account</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>New family account created for independent child</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>Completed Path B direct registration</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>1. In admin /admin/families, search by contact email or name</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>New family account exists with registration_path = child_direct</v>
       </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
       <c r="H7" t="str">
         <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:J16"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="38.83203125" customWidth="1"/>
-    <col min="4" max="4" width="32.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
     <col min="6" max="6" width="48.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="48.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2384,27 +2578,30 @@
         <v>Test ID</v>
       </c>
       <c r="B1" t="str">
+        <v>Tester</v>
+      </c>
+      <c r="C1" t="str">
         <v>Category</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Test Case</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Pre-conditions</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Steps</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Expected Behaviour</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Actual Behaviour</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Pass / Fail</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -2413,29 +2610,32 @@
         <v>INV-001</v>
       </c>
       <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
         <v>Admin — generate token</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Admin generates child_invite token</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Signed in as super_admin; on /admin/families</v>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
+      <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Find a family account
 2. Click "Invite child"
 3. Copy generated URL</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Token created in zawaaj_invite_tokens with purpose=child_invite; URL displayed</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v/>
       </c>
     </row>
@@ -2444,29 +2644,32 @@
         <v>INV-002</v>
       </c>
       <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
         <v>Admin — generate token</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Admin generates guardian_invite token</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Signed in as super_admin</v>
       </c>
-      <c r="E3" t="str" xml:space="preserve">
+      <c r="F3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Find a family account
 2. Click "Invite guardian"
 3. Copy generated URL</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>Token created with purpose=guardian_invite; URL displayed</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
       <c r="H3" t="str">
         <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v/>
       </c>
     </row>
@@ -2475,28 +2678,31 @@
         <v>INV-003</v>
       </c>
       <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
         <v>Admin — email token</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Admin emails invite token to candidate</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Token generated; candidate email on file</v>
       </c>
-      <c r="E4" t="str" xml:space="preserve">
+      <c r="F4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. After generating token URL
 2. Click "✉ Email invite to [email]"</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Email sent to candidate with registration link; "Email sent" confirmation shown</v>
       </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
         <v/>
       </c>
     </row>
@@ -2505,27 +2711,30 @@
         <v>INV-004</v>
       </c>
       <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
         <v>Token validation</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>Valid token accepted on /register/child page</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>Valid unexpired token URL</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>1. Open /register/child?token=&lt;valid_token&gt;</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>Gold "Invited registration" badge shown; guardian step skipped; pre-filled fields visible</v>
       </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
       <c r="H5" t="str">
         <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v/>
       </c>
     </row>
@@ -2534,27 +2743,30 @@
         <v>INV-005</v>
       </c>
       <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
         <v>Token validation</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>Expired token shows error</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>Token older than 7 days</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>1. Open /register/child?token=&lt;expired_token&gt;</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>Error screen: "This invitation has expired"; link to request new one</v>
       </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
         <v/>
       </c>
     </row>
@@ -2563,27 +2775,30 @@
         <v>INV-006</v>
       </c>
       <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
         <v>Token validation</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>Already-used token shows error</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>Token previously used (accepted_at set)</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>1. Open /register/child?token=&lt;used_token&gt;</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>Error screen: "This invitation has already been used"</v>
       </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
       <c r="H7" t="str">
         <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
         <v/>
       </c>
     </row>
@@ -2592,27 +2807,30 @@
         <v>INV-007</v>
       </c>
       <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
         <v>Token validation</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>Invalid/nonexistent token shows error</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>Made-up token string</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>1. Open /register/child?token=FAKEXXX</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>Error screen: "Invalid invitation link"</v>
       </c>
-      <c r="G8" t="str">
-        <v/>
-      </c>
       <c r="H8" t="str">
         <v/>
       </c>
       <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
         <v/>
       </c>
     </row>
@@ -2621,28 +2839,31 @@
         <v>INV-008</v>
       </c>
       <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
         <v>Step skipping</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>Guardian step skipped when token present</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>Valid token accepted</v>
       </c>
-      <c r="E9" t="str" xml:space="preserve">
+      <c r="F9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Step through form with token
 2. Observe step count</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>Guardian details step (step 4) not shown; EFFECTIVE_TOTAL = 7 steps total</v>
       </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
       <c r="H9" t="str">
         <v/>
       </c>
       <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
         <v/>
       </c>
     </row>
@@ -2651,27 +2872,30 @@
         <v>INV-009</v>
       </c>
       <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
         <v>Step skipping</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>Pre-filled guardian fields from token</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>Token contains candidate name and email</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>1. Open form with valid token</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>Email field pre-filled from token; candidate name pre-filled if stored</v>
       </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
       <c r="H10" t="str">
         <v/>
       </c>
       <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
         <v/>
       </c>
     </row>
@@ -2680,28 +2904,31 @@
         <v>INV-010</v>
       </c>
       <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
         <v>Auto-linkage</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>Profile linked to existing family account on submit</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>Valid token; completed all steps</v>
       </c>
-      <c r="E11" t="str" xml:space="preserve">
+      <c r="F11" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Complete registration with valid token
 2. Submit</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>New profile created; family_account_id set to existing family account; NO new family account created</v>
       </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
       <c r="H11" t="str">
         <v/>
       </c>
       <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
         <v/>
       </c>
     </row>
@@ -2710,28 +2937,31 @@
         <v>INV-011</v>
       </c>
       <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
         <v>Auto-linkage</v>
       </c>
-      <c r="C12" t="str">
+      <c r="D12" t="str">
         <v>Token marked as used after successful registration</v>
       </c>
-      <c r="D12" t="str">
+      <c r="E12" t="str">
         <v>Valid token; registration completed</v>
       </c>
-      <c r="E12" t="str" xml:space="preserve">
+      <c r="F12" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Complete registration
 2. Try to use same token URL again</v>
       </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
         <v>Token accepted_at is now set; second attempt shows "already used" error</v>
       </c>
-      <c r="G12" t="str">
-        <v/>
-      </c>
       <c r="H12" t="str">
         <v/>
       </c>
       <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
         <v/>
       </c>
     </row>
@@ -2740,28 +2970,31 @@
         <v>INV-012</v>
       </c>
       <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
         <v>Auto-linkage</v>
       </c>
-      <c r="C13" t="str">
+      <c r="D13" t="str">
         <v>Admin can see linked profile under family account</v>
       </c>
-      <c r="D13" t="str">
+      <c r="E13" t="str">
         <v>Registration completed via invite token</v>
       </c>
-      <c r="E13" t="str" xml:space="preserve">
+      <c r="F13" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Go to /admin/families
 2. Open the family account that issued the token</v>
       </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
         <v>New member profile appears under family account members list</v>
       </c>
-      <c r="G13" t="str">
-        <v/>
-      </c>
       <c r="H13" t="str">
         <v/>
       </c>
       <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
         <v/>
       </c>
     </row>
@@ -2770,27 +3003,30 @@
         <v>INV-013</v>
       </c>
       <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
         <v>Admin — families view</v>
       </c>
-      <c r="C14" t="str">
+      <c r="D14" t="str">
         <v>Families page lists all family accounts</v>
       </c>
-      <c r="D14" t="str">
+      <c r="E14" t="str">
         <v>Signed in as super_admin</v>
       </c>
-      <c r="E14" t="str">
+      <c r="F14" t="str">
         <v>1. Navigate to /admin/families</v>
       </c>
-      <c r="F14" t="str">
+      <c r="G14" t="str">
         <v>All family accounts listed with contact info, member count, registration path</v>
       </c>
-      <c r="G14" t="str">
-        <v/>
-      </c>
       <c r="H14" t="str">
         <v/>
       </c>
       <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
         <v/>
       </c>
     </row>
@@ -2799,27 +3035,30 @@
         <v>INV-014</v>
       </c>
       <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
         <v>Admin — families view</v>
       </c>
-      <c r="C15" t="str">
+      <c r="D15" t="str">
         <v>Filter families by registration path</v>
       </c>
-      <c r="D15" t="str">
+      <c r="E15" t="str">
         <v>On /admin/families</v>
       </c>
-      <c r="E15" t="str">
+      <c r="F15" t="str">
         <v>1. Apply filter for "direct" or "child_direct"</v>
       </c>
-      <c r="F15" t="str">
+      <c r="G15" t="str">
         <v>List updates to show only matching families</v>
       </c>
-      <c r="G15" t="str">
-        <v/>
-      </c>
       <c r="H15" t="str">
         <v/>
       </c>
       <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
         <v/>
       </c>
     </row>
@@ -2828,50 +3067,54 @@
         <v>INV-015</v>
       </c>
       <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
         <v>Admin — families view</v>
       </c>
-      <c r="C16" t="str">
+      <c r="D16" t="str">
         <v>Search families by name or email</v>
       </c>
-      <c r="D16" t="str">
+      <c r="E16" t="str">
         <v>On /admin/families</v>
       </c>
-      <c r="E16" t="str">
+      <c r="F16" t="str">
         <v>1. Type in search box</v>
       </c>
-      <c r="F16" t="str">
+      <c r="G16" t="str">
         <v>Results filter to matching families</v>
       </c>
-      <c r="G16" t="str">
-        <v/>
-      </c>
       <c r="H16" t="str">
         <v/>
       </c>
       <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="38.83203125" customWidth="1"/>
-    <col min="4" max="4" width="32.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
     <col min="6" max="6" width="48.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="48.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2879,27 +3122,30 @@
         <v>Test ID</v>
       </c>
       <c r="B1" t="str">
+        <v>Tester</v>
+      </c>
+      <c r="C1" t="str">
         <v>Category</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Test Case</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Pre-conditions</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Steps</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Expected Behaviour</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Actual Behaviour</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Pass / Fail</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -2908,28 +3154,31 @@
         <v>EVT-001</v>
       </c>
       <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
         <v>Admin events</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Admin can access /admin/events</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Signed in as super_admin</v>
       </c>
-      <c r="E2" t="str" xml:space="preserve">
+      <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click "Events" in admin sidebar
 2. Or navigate to /admin/events</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Events management page loads with list of all events</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
       <c r="H2" t="str">
         <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v/>
       </c>
     </row>
@@ -2938,30 +3187,33 @@
         <v>EVT-002</v>
       </c>
       <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
         <v>Admin events</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Create a new upcoming event</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>On /admin/events</v>
       </c>
-      <c r="E3" t="str" xml:space="preserve">
+      <c r="F3" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click "+ New event"
 2. Enter title, date, location, registration URL
 3. Set status to Upcoming
 4. Click Create</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>Event created; appears in list with Upcoming badge; visible to members on /events</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
       <c r="H3" t="str">
         <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v/>
       </c>
     </row>
@@ -2970,29 +3222,32 @@
         <v>EVT-003</v>
       </c>
       <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
         <v>Admin events</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Create event without registration URL</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>On /admin/events; new event modal open</v>
       </c>
-      <c r="E4" t="str" xml:space="preserve">
+      <c r="F4" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Enter title and date
 2. Leave registration URL blank
 3. Create</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>Event created; member-facing page shows "Registration details coming soon"</v>
       </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
       <c r="H4" t="str">
         <v/>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
         <v/>
       </c>
     </row>
@@ -3001,29 +3256,32 @@
         <v>EVT-004</v>
       </c>
       <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
         <v>Admin events</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>Edit an existing event</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>Event exists in list</v>
       </c>
-      <c r="E5" t="str" xml:space="preserve">
+      <c r="F5" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click Edit on an event
 2. Update location or status
 3. Save</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>Changes saved; event card updated immediately in admin list</v>
       </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
       <c r="H5" t="str">
         <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v/>
       </c>
     </row>
@@ -3032,29 +3290,32 @@
         <v>EVT-005</v>
       </c>
       <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
         <v>Admin events</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>Mark event as Ended</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>Upcoming event exists</v>
       </c>
-      <c r="E6" t="str" xml:space="preserve">
+      <c r="F6" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Edit event
 2. Change status to "Ended"
 3. Save</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>Status badge changes to Ended; event no longer appears in members' upcoming section</v>
       </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
       <c r="H6" t="str">
         <v/>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
         <v/>
       </c>
     </row>
@@ -3063,29 +3324,32 @@
         <v>EVT-006</v>
       </c>
       <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
         <v>Admin events</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>Enable show_in_history for past event</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>Event with status = ended</v>
       </c>
-      <c r="E7" t="str" xml:space="preserve">
+      <c r="F7" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Edit event
 2. Check "Show in past events history"
 3. Save</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>Event appears in "Past events" section on member-facing /events page</v>
       </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
       <c r="H7" t="str">
         <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
         <v/>
       </c>
     </row>
@@ -3094,29 +3358,32 @@
         <v>EVT-007</v>
       </c>
       <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
         <v>Admin events</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>Add attendance note to past event</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>Ended event</v>
       </c>
-      <c r="E8" t="str" xml:space="preserve">
+      <c r="F8" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Edit event
 2. Add attendance note (e.g. "47 attendees")
 3. Save</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>Note displayed on past event card for members</v>
       </c>
-      <c r="G8" t="str">
-        <v/>
-      </c>
       <c r="H8" t="str">
         <v/>
       </c>
       <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
         <v/>
       </c>
     </row>
@@ -3125,28 +3392,31 @@
         <v>EVT-008</v>
       </c>
       <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
         <v>Admin events</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>Archive an event</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>Any non-archived event</v>
       </c>
-      <c r="E9" t="str" xml:space="preserve">
+      <c r="F9" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Click Archive button
 2. Confirm prompt</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>Event status → archived; disappears from member view; still visible in admin list with "Archived" filter</v>
       </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
       <c r="H9" t="str">
         <v/>
       </c>
       <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
         <v/>
       </c>
     </row>
@@ -3155,27 +3425,30 @@
         <v>EVT-009</v>
       </c>
       <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
         <v>Admin events</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>Filter events by status in admin</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>Multiple events in different statuses</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>1. Click Upcoming / Ended / Archived filter tabs</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>List filters to show only matching events</v>
       </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
       <c r="H10" t="str">
         <v/>
       </c>
       <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
         <v/>
       </c>
     </row>
@@ -3184,28 +3457,31 @@
         <v>EVT-010</v>
       </c>
       <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
         <v>Member events</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>Member sees upcoming events</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>Upcoming event exists with show_in_history or status=upcoming</v>
       </c>
-      <c r="E11" t="str" xml:space="preserve">
+      <c r="F11" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Sign in as member
 2. Navigate to /events</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>Upcoming event card with gold left border, date, location, register button</v>
       </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
       <c r="H11" t="str">
         <v/>
       </c>
       <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
         <v/>
       </c>
     </row>
@@ -3214,28 +3490,31 @@
         <v>EVT-011</v>
       </c>
       <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
         <v>Member events</v>
       </c>
-      <c r="C12" t="str">
+      <c r="D12" t="str">
         <v>Member sees past events</v>
       </c>
-      <c r="D12" t="str">
+      <c r="E12" t="str">
         <v>Event with status=ended and show_in_history=true</v>
       </c>
-      <c r="E12" t="str" xml:space="preserve">
+      <c r="F12" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to /events
 2. Scroll to past events</v>
       </c>
-      <c r="F12" t="str">
+      <c r="G12" t="str">
         <v>Past event listed with date and attendance note if set</v>
       </c>
-      <c r="G12" t="str">
-        <v/>
-      </c>
       <c r="H12" t="str">
         <v/>
       </c>
       <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
         <v/>
       </c>
     </row>
@@ -3244,33 +3523,36 @@
         <v>EVT-012</v>
       </c>
       <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
         <v>Member events</v>
       </c>
-      <c r="C13" t="str">
+      <c r="D13" t="str">
         <v>Archived events hidden from members</v>
       </c>
-      <c r="D13" t="str">
+      <c r="E13" t="str">
         <v>Event with status=archived</v>
       </c>
-      <c r="E13" t="str">
+      <c r="F13" t="str">
         <v>1. Navigate to /events</v>
       </c>
-      <c r="F13" t="str">
+      <c r="G13" t="str">
         <v>Archived event not visible anywhere on member events page</v>
       </c>
-      <c r="G13" t="str">
-        <v/>
-      </c>
       <c r="H13" t="str">
         <v/>
       </c>
       <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: add GDPR privacy & data rights sheet to test cases (106 total)
Sheet 7 covers cookie notice, privacy policy, terms GDPR clauses,
data rights portal (export, rectify, erase, cancel, history) — 20 new cases.
Plain non-technical language throughout for non-IT testers.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases/Zawaaj_Test_Cases.xlsx
+++ b/test-cases/Zawaaj_Test_Cases.xlsx
@@ -9,6 +9,7 @@
     <sheet name="4. Child Path B (Direct)" sheetId="4" r:id="rId4"/>
     <sheet name="5. Invite Token Auto-Linkage" sheetId="5" r:id="rId5"/>
     <sheet name="6. Admin Events CRUD" sheetId="6" r:id="rId6"/>
+    <sheet name="7. Privacy &amp; Data Rights" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -3555,4 +3556,717 @@
     <ignoredError numberStoredAsText="1" sqref="A1:J13"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J21"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
+    <col min="6" max="6" width="48.83203125" customWidth="1"/>
+    <col min="7" max="7" width="48.83203125" customWidth="1"/>
+    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Test ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Tester</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Test Case</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Pre-conditions</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Steps</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Expected Behaviour</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Actual Behaviour</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Pass / Fail</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>GDPR-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>Cookie Notice</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Cookie notice appears on first visit</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Fresh browser / cleared browser storage (or use private/incognito window)</v>
+      </c>
+      <c r="F2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open zawaaj.uk in a new private/incognito window
+2. Wait for the page to fully load</v>
+      </c>
+      <c r="G2" t="str">
+        <v>A small notice bar appears at the bottom of the screen saying the site uses strictly necessary cookies only, with a "Got it" button and a link to the Privacy Policy</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>GDPR-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>Cookie Notice</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Cookie notice disappears after clicking "Got it"</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Cookie notice is visible on screen</v>
+      </c>
+      <c r="F3" t="str">
+        <v>1. Click the "Got it" button on the cookie notice</v>
+      </c>
+      <c r="G3" t="str">
+        <v>The notice bar closes immediately and does not reappear when navigating to other pages</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>GDPR-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v>Cookie Notice</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Cookie notice does not reappear on return visit</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Already clicked "Got it" on this device/browser</v>
+      </c>
+      <c r="F4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Close the browser tab
+2. Open zawaaj.uk again in the same browser (not incognito)</v>
+      </c>
+      <c r="G4" t="str">
+        <v>The cookie notice does not appear — it stays dismissed</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>GDPR-004</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v>Privacy Policy</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Privacy Policy page is publicly accessible (no login needed)</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Not logged in</v>
+      </c>
+      <c r="F5" t="str">
+        <v>1. Go to zawaaj.uk/privacy</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Full Privacy Policy page loads — no login required; page shows Ingenious Education Ltd as Data Controller and Zawaaj as Data Processor</v>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>GDPR-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v>Privacy Policy</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Privacy Policy link in cookie notice works</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Cookie notice visible on screen</v>
+      </c>
+      <c r="F6" t="str">
+        <v>1. Click the "Privacy Policy" link in the cookie notice</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Navigates to /privacy — Privacy Policy page loads correctly</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>GDPR-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v>Privacy Policy</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Privacy link in sidebar works for logged-in members</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Signed in as an approved member</v>
+      </c>
+      <c r="F7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Look at the left-hand sidebar
+2. Click "Privacy" (below Help centre)</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Navigates to /privacy — Privacy Policy page loads</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>GDPR-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v>Terms &amp; Conditions</v>
+      </c>
+      <c r="D8" t="str">
+        <v>GDPR clauses visible on Terms page</v>
+      </c>
+      <c r="E8" t="str">
+        <v>None</v>
+      </c>
+      <c r="F8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Go to zawaaj.uk/terms
+2. Scroll to clauses 11–14</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Four new sections visible: "Data Controller &amp; Processor", "Your Data Protection Rights", "Cookies", and "Changes to These Terms"</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>GDPR-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v>Terms &amp; Conditions</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Privacy Policy link at bottom of Terms page works</v>
+      </c>
+      <c r="E9" t="str">
+        <v>On /terms page</v>
+      </c>
+      <c r="F9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Scroll to the very bottom of the Terms page
+2. Click "Privacy Policy →"</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Navigates to /privacy — Privacy Policy loads</v>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>GDPR-009</v>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v>Data Rights Portal</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Data rights page requires login</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Not logged in</v>
+      </c>
+      <c r="F10" t="str">
+        <v>1. Go to zawaaj.uk/privacy/rights</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Redirected to /login — cannot access the data rights page without being signed in</v>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>GDPR-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v>Data Rights Portal</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Data rights portal loads for logged-in member</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Signed in as an approved member</v>
+      </c>
+      <c r="F11" t="str">
+        <v>1. Go to zawaaj.uk/privacy/rights  (or click Privacy in sidebar, then click "Manage your data rights")</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Page loads with five tabs: Overview, Request my data, Correct my data, Delete my account, Request history</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>GDPR-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v>Data Rights Portal</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Overview tab shows action cards</v>
+      </c>
+      <c r="E12" t="str">
+        <v>On /privacy/rights — Overview tab</v>
+      </c>
+      <c r="F12" t="str">
+        <v>1. Check the Overview tab</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Four action cards visible: "Download my data", "Correct my data", "Delete my account", "View request history"</v>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>GDPR-012</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v>Request My Data</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Member can request a copy of their data</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Signed in as member; on /privacy/rights — "Request my data" tab; no export request in the last 30 days</v>
+      </c>
+      <c r="F13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click the "Request my data" tab
+2. Click "Send me my data"</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Success message shown — "We've sent a copy of your data to your registered email address"; an email arrives with a downloadable file attached</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>GDPR-013</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v>Request My Data</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Second export request within 30 days is blocked</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Already submitted an export request within the last 30 days</v>
+      </c>
+      <c r="F14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Go to "Request my data" tab
+2. Try to click "Send me my data" again</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Message shown explaining that only one export is allowed every 30 days; the button is disabled or shows when the next request can be made</v>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>GDPR-014</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v>Correct My Data</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Member can submit a correction request</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Signed in; on "Correct my data" tab; fewer than 3 pending correction requests</v>
+      </c>
+      <c r="F15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click the "Correct my data" tab
+2. Select a field (e.g. Location)
+3. Enter the correct value
+4. Add a brief reason
+5. Click Submit</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Success message shown — request submitted; appears in Request history with status "Pending"</v>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>GDPR-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v>Correct My Data</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Cannot have more than 3 open correction requests at once</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Already have 3 correction requests with status "Pending"</v>
+      </c>
+      <c r="F16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Go to "Correct my data" tab
+2. Try to submit another correction</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Error message shown — cannot submit more than 3 correction requests at a time; told to wait for existing ones to be processed</v>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>GDPR-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v>Delete My Account</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Delete account requires typing a confirmation phrase</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Signed in; on "Delete my account" tab</v>
+      </c>
+      <c r="F17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click "Delete my account" tab
+2. Check the confirmation checkbox
+3. Leave the confirmation phrase box empty
+4. Try to click "Request account deletion"</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Button remains inactive or shows an error — the exact phrase "DELETE MY ACCOUNT" must be typed before the request can be submitted</v>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>GDPR-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v>Delete My Account</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Delete account request submitted successfully</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Signed in; on "Delete my account" tab</v>
+      </c>
+      <c r="F18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Check the confirmation checkbox
+2. Type DELETE MY ACCOUNT in the text box (exactly as shown)
+3. Click "Request account deletion"</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Success message shown — account is scheduled for deletion in 7 days; profile immediately disappears from the member directory; a cancellation link is sent to the registered email address</v>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>GDPR-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v>Delete My Account</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Member can cancel their deletion request via email link</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Deletion request submitted; cancellation email received</v>
+      </c>
+      <c r="F19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open the cancellation email
+2. Click "Cancel my deletion request"</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Browser opens with a message confirming the deletion has been cancelled; profile is restored (status set to paused — no longer in the browse directory but account is active)</v>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>GDPR-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v>Request History</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Submitted requests appear in history tab</v>
+      </c>
+      <c r="E20" t="str">
+        <v>At least one request has been submitted (export, correction, or deletion)</v>
+      </c>
+      <c r="F20" t="str">
+        <v>1. Go to "Request history" tab</v>
+      </c>
+      <c r="G20" t="str">
+        <v>All past requests listed with type, date submitted, and current status (Pending / Completed / Cancelled)</v>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>GDPR-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v>Request History</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Empty history shows friendly message</v>
+      </c>
+      <c r="E21" t="str">
+        <v>No requests have ever been submitted</v>
+      </c>
+      <c r="F21" t="str">
+        <v>1. Go to "Request history" tab</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Message shown: "No requests yet" or similar — no blank/broken table</v>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:J21"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: move data rights self-serve into Settings → Privacy tab
Members can now download their data and delete their account directly
from Settings → Privacy tab, without needing to know about /privacy/rights.
- Download data: one-click with 30-day rate-limit feedback inline
- Delete account: confirmation checkbox + phrase input + 7-day cooling-off
- /privacy/rights retained for full request history and correction requests
- Test cases updated to reflect Settings as the primary self-serve path

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test-cases/Zawaaj_Test_Cases.xlsx
+++ b/test-cases/Zawaaj_Test_Cases.xlsx
@@ -3867,7 +3867,7 @@
         <v/>
       </c>
     </row>
-    <row r="10">
+    <row r="10" xml:space="preserve">
       <c r="A10" t="str">
         <v>GDPR-009</v>
       </c>
@@ -3875,19 +3875,20 @@
         <v/>
       </c>
       <c r="C10" t="str">
-        <v>Data Rights Portal</v>
+        <v>Settings — Privacy tab</v>
       </c>
       <c r="D10" t="str">
-        <v>Data rights page requires login</v>
+        <v>Privacy tab visible in account settings</v>
       </c>
       <c r="E10" t="str">
-        <v>Not logged in</v>
-      </c>
-      <c r="F10" t="str">
-        <v>1. Go to zawaaj.uk/privacy/rights</v>
+        <v>Signed in as an approved member</v>
+      </c>
+      <c r="F10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click "Settings" in the left-hand sidebar
+2. Click the "Privacy" tab at the top of the page</v>
       </c>
       <c r="G10" t="str">
-        <v>Redirected to /login — cannot access the data rights page without being signed in</v>
+        <v>Privacy tab content loads showing: data protection summary, "Download a copy of my data" section, "Delete my account" section, and links to Privacy Policy and Terms</v>
       </c>
       <c r="H10" t="str">
         <v/>
@@ -3899,7 +3900,7 @@
         <v/>
       </c>
     </row>
-    <row r="11">
+    <row r="11" xml:space="preserve">
       <c r="A11" t="str">
         <v>GDPR-010</v>
       </c>
@@ -3907,19 +3908,20 @@
         <v/>
       </c>
       <c r="C11" t="str">
-        <v>Data Rights Portal</v>
+        <v>Settings — Privacy tab</v>
       </c>
       <c r="D11" t="str">
-        <v>Data rights portal loads for logged-in member</v>
+        <v>Member can request a copy of their data from Settings</v>
       </c>
       <c r="E11" t="str">
-        <v>Signed in as an approved member</v>
-      </c>
-      <c r="F11" t="str">
-        <v>1. Go to zawaaj.uk/privacy/rights  (or click Privacy in sidebar, then click "Manage your data rights")</v>
+        <v>Signed in; on Settings → Privacy tab; no export request submitted in the last 30 days</v>
+      </c>
+      <c r="F11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Go to Settings → Privacy tab
+2. Click "Send me a copy of my data"</v>
       </c>
       <c r="G11" t="str">
-        <v>Page loads with five tabs: Overview, Request my data, Correct my data, Delete my account, Request history</v>
+        <v>Button shows "Sending…" briefly; then a green success message appears: "Done — a copy of your data has been sent to your registered email address." An email arrives with the data attached.</v>
       </c>
       <c r="H11" t="str">
         <v/>
@@ -3931,7 +3933,7 @@
         <v/>
       </c>
     </row>
-    <row r="12">
+    <row r="12" xml:space="preserve">
       <c r="A12" t="str">
         <v>GDPR-011</v>
       </c>
@@ -3939,19 +3941,20 @@
         <v/>
       </c>
       <c r="C12" t="str">
-        <v>Data Rights Portal</v>
+        <v>Settings — Privacy tab</v>
       </c>
       <c r="D12" t="str">
-        <v>Overview tab shows action cards</v>
+        <v>Second export request within 30 days is blocked</v>
       </c>
       <c r="E12" t="str">
-        <v>On /privacy/rights — Overview tab</v>
-      </c>
-      <c r="F12" t="str">
-        <v>1. Check the Overview tab</v>
+        <v>Already requested a data copy within the last 30 days</v>
+      </c>
+      <c r="F12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Go to Settings → Privacy tab
+2. Click "Send me a copy of my data" again</v>
       </c>
       <c r="G12" t="str">
-        <v>Four action cards visible: "Download my data", "Correct my data", "Delete my account", "View request history"</v>
+        <v>An error message appears explaining that only one data export is allowed every 30 days</v>
       </c>
       <c r="H12" t="str">
         <v/>
@@ -3971,20 +3974,20 @@
         <v/>
       </c>
       <c r="C13" t="str">
-        <v>Request My Data</v>
+        <v>Settings — Privacy tab</v>
       </c>
       <c r="D13" t="str">
-        <v>Member can request a copy of their data</v>
+        <v>Delete account button appears in Settings</v>
       </c>
       <c r="E13" t="str">
-        <v>Signed in as member; on /privacy/rights — "Request my data" tab; no export request in the last 30 days</v>
+        <v>Signed in; on Settings → Privacy tab</v>
       </c>
       <c r="F13" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Click the "Request my data" tab
-2. Click "Send me my data"</v>
+        <v xml:space="preserve">1. Go to Settings → Privacy tab
+2. Scroll to "Delete my account" section</v>
       </c>
       <c r="G13" t="str">
-        <v>Success message shown — "We've sent a copy of your data to your registered email address"; an email arrives with a downloadable file attached</v>
+        <v>"Delete my account" button visible with a brief explanation of the 7-day waiting period</v>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -4004,20 +4007,21 @@
         <v/>
       </c>
       <c r="C14" t="str">
-        <v>Request My Data</v>
+        <v>Delete My Account</v>
       </c>
       <c r="D14" t="str">
-        <v>Second export request within 30 days is blocked</v>
+        <v>Delete account requires ticking confirmation box and typing a phrase</v>
       </c>
       <c r="E14" t="str">
-        <v>Already submitted an export request within the last 30 days</v>
+        <v>Signed in; on Settings → Privacy tab; "Delete my account" section visible</v>
       </c>
       <c r="F14" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Go to "Request my data" tab
-2. Try to click "Send me my data" again</v>
+        <v xml:space="preserve">1. Click "Delete my account"
+2. Leave the confirmation box unticked and the text box empty
+3. Try to click "Request account deletion"</v>
       </c>
       <c r="G14" t="str">
-        <v>Message shown explaining that only one export is allowed every 30 days; the button is disabled or shows when the next request can be made</v>
+        <v>The "Request account deletion" button is greyed out and cannot be clicked — both the tick box and the exact phrase must be completed first</v>
       </c>
       <c r="H14" t="str">
         <v/>
@@ -4037,23 +4041,22 @@
         <v/>
       </c>
       <c r="C15" t="str">
-        <v>Correct My Data</v>
+        <v>Delete My Account</v>
       </c>
       <c r="D15" t="str">
-        <v>Member can submit a correction request</v>
+        <v>Delete account submitted successfully</v>
       </c>
       <c r="E15" t="str">
-        <v>Signed in; on "Correct my data" tab; fewer than 3 pending correction requests</v>
+        <v>Signed in; on Settings → Privacy tab; "Delete my account" section visible</v>
       </c>
       <c r="F15" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Click the "Correct my data" tab
-2. Select a field (e.g. Location)
-3. Enter the correct value
-4. Add a brief reason
-5. Click Submit</v>
+        <v xml:space="preserve">1. Click "Delete my account"
+2. Tick the confirmation box
+3. Type DELETE MY ACCOUNT in the text box exactly as shown
+4. Click "Request account deletion"</v>
       </c>
       <c r="G15" t="str">
-        <v>Success message shown — request submitted; appears in Request history with status "Pending"</v>
+        <v>Red confirmation message shown: "Deletion request submitted — your profile has been removed from the directory. Account will be permanently deleted in 7 days." A cancellation email is sent to the registered address.</v>
       </c>
       <c r="H15" t="str">
         <v/>
@@ -4073,20 +4076,20 @@
         <v/>
       </c>
       <c r="C16" t="str">
-        <v>Correct My Data</v>
+        <v>Delete My Account</v>
       </c>
       <c r="D16" t="str">
-        <v>Cannot have more than 3 open correction requests at once</v>
+        <v>Cancel button during deletion flow works</v>
       </c>
       <c r="E16" t="str">
-        <v>Already have 3 correction requests with status "Pending"</v>
+        <v>Clicked "Delete my account" and confirmation form is showing</v>
       </c>
       <c r="F16" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Go to "Correct my data" tab
-2. Try to submit another correction</v>
+        <v xml:space="preserve">1. Click "Delete my account" to open the form
+2. Click "Cancel"</v>
       </c>
       <c r="G16" t="str">
-        <v>Error message shown — cannot submit more than 3 correction requests at a time; told to wait for existing ones to be processed</v>
+        <v>Form closes; returns to the normal privacy tab view; nothing is deleted</v>
       </c>
       <c r="H16" t="str">
         <v/>
@@ -4109,19 +4112,17 @@
         <v>Delete My Account</v>
       </c>
       <c r="D17" t="str">
-        <v>Delete account requires typing a confirmation phrase</v>
+        <v>Member can cancel their deletion request via email link</v>
       </c>
       <c r="E17" t="str">
-        <v>Signed in; on "Delete my account" tab</v>
+        <v>Deletion request submitted; cancellation email received in inbox</v>
       </c>
       <c r="F17" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Click "Delete my account" tab
-2. Check the confirmation checkbox
-3. Leave the confirmation phrase box empty
-4. Try to click "Request account deletion"</v>
+        <v xml:space="preserve">1. Open the cancellation email
+2. Click the cancellation link in the email</v>
       </c>
       <c r="G17" t="str">
-        <v>Button remains inactive or shows an error — the exact phrase "DELETE MY ACCOUNT" must be typed before the request can be submitted</v>
+        <v>A webpage opens confirming the deletion has been cancelled; the account is restored to a paused state (profile is not in the directory but the account is still active)</v>
       </c>
       <c r="H17" t="str">
         <v/>
@@ -4141,21 +4142,24 @@
         <v/>
       </c>
       <c r="C18" t="str">
-        <v>Delete My Account</v>
+        <v>Correct My Data</v>
       </c>
       <c r="D18" t="str">
-        <v>Delete account request submitted successfully</v>
+        <v>Member can submit a correction request via the data rights portal</v>
       </c>
       <c r="E18" t="str">
-        <v>Signed in; on "Delete my account" tab</v>
+        <v>Signed in; fewer than 3 pending correction requests already open</v>
       </c>
       <c r="F18" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Check the confirmation checkbox
-2. Type DELETE MY ACCOUNT in the text box (exactly as shown)
-3. Click "Request account deletion"</v>
+        <v xml:space="preserve">1. Go to zawaaj.uk/privacy/rights
+2. Click the "Correct my data" tab
+3. Select the field to correct (e.g. Location)
+4. Enter the correct value
+5. Add a short explanation
+6. Click Submit</v>
       </c>
       <c r="G18" t="str">
-        <v>Success message shown — account is scheduled for deletion in 7 days; profile immediately disappears from the member directory; a cancellation link is sent to the registered email address</v>
+        <v>Success message shown — request has been submitted; visible in the Request History tab with status "Pending"; admin will review and make the correction</v>
       </c>
       <c r="H18" t="str">
         <v/>
@@ -4175,20 +4179,20 @@
         <v/>
       </c>
       <c r="C19" t="str">
-        <v>Delete My Account</v>
+        <v>Correct My Data</v>
       </c>
       <c r="D19" t="str">
-        <v>Member can cancel their deletion request via email link</v>
+        <v>Cannot have more than 3 open correction requests at once</v>
       </c>
       <c r="E19" t="str">
-        <v>Deletion request submitted; cancellation email received</v>
+        <v>Already have 3 correction requests with status "Pending"</v>
       </c>
       <c r="F19" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Open the cancellation email
-2. Click "Cancel my deletion request"</v>
+        <v xml:space="preserve">1. Go to zawaaj.uk/privacy/rights → "Correct my data" tab
+2. Try to submit another correction</v>
       </c>
       <c r="G19" t="str">
-        <v>Browser opens with a message confirming the deletion has been cancelled; profile is restored (status set to paused — no longer in the browse directory but account is active)</v>
+        <v>Error message shown — cannot submit more than 3 correction requests at a time; advised to wait for existing requests to be resolved first</v>
       </c>
       <c r="H19" t="str">
         <v/>
@@ -4200,7 +4204,7 @@
         <v/>
       </c>
     </row>
-    <row r="20">
+    <row r="20" xml:space="preserve">
       <c r="A20" t="str">
         <v>GDPR-019</v>
       </c>
@@ -4208,19 +4212,20 @@
         <v/>
       </c>
       <c r="C20" t="str">
-        <v>Request History</v>
+        <v>Data Rights History</v>
       </c>
       <c r="D20" t="str">
-        <v>Submitted requests appear in history tab</v>
+        <v>Request history accessible at /privacy/rights</v>
       </c>
       <c r="E20" t="str">
-        <v>At least one request has been submitted (export, correction, or deletion)</v>
-      </c>
-      <c r="F20" t="str">
-        <v>1. Go to "Request history" tab</v>
+        <v>Signed in; at least one data request has been submitted</v>
+      </c>
+      <c r="F20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Go to zawaaj.uk/privacy/rights
+2. Click "Request history" tab</v>
       </c>
       <c r="G20" t="str">
-        <v>All past requests listed with type, date submitted, and current status (Pending / Completed / Cancelled)</v>
+        <v>All past data requests listed with type (e.g. Data export, Correction, Deletion), date submitted, and current status</v>
       </c>
       <c r="H20" t="str">
         <v/>
@@ -4232,7 +4237,7 @@
         <v/>
       </c>
     </row>
-    <row r="21">
+    <row r="21" xml:space="preserve">
       <c r="A21" t="str">
         <v>GDPR-020</v>
       </c>
@@ -4240,19 +4245,20 @@
         <v/>
       </c>
       <c r="C21" t="str">
-        <v>Request History</v>
+        <v>Data Rights History</v>
       </c>
       <c r="D21" t="str">
-        <v>Empty history shows friendly message</v>
+        <v>Empty history shows a friendly message</v>
       </c>
       <c r="E21" t="str">
-        <v>No requests have ever been submitted</v>
-      </c>
-      <c r="F21" t="str">
-        <v>1. Go to "Request history" tab</v>
+        <v>Signed in; no data requests have ever been submitted</v>
+      </c>
+      <c r="F21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Go to zawaaj.uk/privacy/rights
+2. Click "Request history" tab</v>
       </c>
       <c r="G21" t="str">
-        <v>Message shown: "No requests yet" or similar — no blank/broken table</v>
+        <v>A message is shown such as "No requests yet" — no blank or broken table</v>
       </c>
       <c r="H21" t="str">
         <v/>

</xml_diff>